<commit_message>
updates to document display
</commit_message>
<xml_diff>
--- a/ABET/DocumentTracker_Assessment.xlsx
+++ b/ABET/DocumentTracker_Assessment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usarmywestpoint-my.sharepoint.com/personal/andrew_biaglow_westpoint_edu/Documents/Documents/GitHub/abiaglow.github.io/ABET/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4C24B4C-F800-408D-BCE3-BAF1805A30FF}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9D051DB-9FF3-4D20-A655-00DD64EDB79A}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-72" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
   </bookViews>
@@ -2782,8 +2782,8 @@
       <c r="J19" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="K19" s="84" t="s">
-        <v>52</v>
+      <c r="K19" s="85" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="3:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update advisory board minutes
</commit_message>
<xml_diff>
--- a/ABET/DocumentTracker_Assessment.xlsx
+++ b/ABET/DocumentTracker_Assessment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usarmywestpoint-my.sharepoint.com/personal/andrew_biaglow_westpoint_edu/Documents/Documents/GitHub/abiaglow.github.io/ABET/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{510FBF87-923A-42C9-BE16-FB452038A73B}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A341C86-E72B-4701-8C4E-954FA9B09F0C}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-72" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
   </bookViews>
@@ -694,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -901,9 +901,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -920,6 +917,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1256,15 +1267,15 @@
     <row r="3" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C3" s="13"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="101" t="s">
+      <c r="E3" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="103"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="100"/>
+      <c r="K3" s="102"/>
     </row>
     <row r="4" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C4" s="14"/>
@@ -1290,15 +1301,15 @@
       <c r="K4" s="15">
         <v>2026</v>
       </c>
-      <c r="N4" s="104" t="s">
+      <c r="N4" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="O4" s="105"/>
+      <c r="O4" s="104"/>
       <c r="P4" s="42"/>
-      <c r="R4" s="104" t="s">
+      <c r="R4" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="S4" s="105"/>
+      <c r="S4" s="104"/>
       <c r="T4" s="42"/>
       <c r="V4" s="54" t="s">
         <v>45</v>
@@ -2391,15 +2402,15 @@
     <row r="3" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C3" s="13"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="101" t="s">
+      <c r="E3" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="103"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="100"/>
+      <c r="K3" s="102"/>
     </row>
     <row r="4" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C4" s="14"/>
@@ -2430,12 +2441,12 @@
       <c r="C5" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="71"/>
+      <c r="D5" s="105"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="71"/>
-      <c r="H5" s="71"/>
-      <c r="I5" s="71"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
       <c r="J5" s="58"/>
       <c r="K5" s="17"/>
     </row>
@@ -2443,20 +2454,20 @@
       <c r="C6" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="71"/>
+      <c r="D6" s="105"/>
       <c r="E6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H6" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I6" s="72" t="s">
+      <c r="F6" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I6" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J6" s="52" t="s">
@@ -2470,20 +2481,20 @@
       <c r="C7" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="71"/>
+      <c r="D7" s="105"/>
       <c r="E7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G7" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I7" s="72" t="s">
+      <c r="F7" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H7" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I7" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J7" s="52" t="s">
@@ -2497,20 +2508,20 @@
       <c r="C8" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="71"/>
+      <c r="D8" s="105"/>
       <c r="E8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F8" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G8" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H8" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8" s="72" t="s">
+      <c r="F8" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H8" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I8" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J8" s="52" t="s">
@@ -2537,7 +2548,7 @@
       <c r="H9" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="I9" s="72" t="s">
+      <c r="I9" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J9" s="63" t="s">
@@ -2575,7 +2586,7 @@
       </c>
     </row>
     <row r="11" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C11" s="100" t="s">
+      <c r="C11" s="99" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="60"/>
@@ -2583,7 +2594,7 @@
       <c r="F11" s="51"/>
       <c r="G11" s="51"/>
       <c r="H11" s="51"/>
-      <c r="I11" s="71"/>
+      <c r="I11" s="105"/>
       <c r="J11" s="58"/>
       <c r="K11" s="17"/>
     </row>
@@ -2595,16 +2606,16 @@
       <c r="E12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F12" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G12" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H12" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I12" s="72" t="s">
+      <c r="F12" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H12" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I12" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J12" s="52" t="s">
@@ -2620,12 +2631,12 @@
       </c>
       <c r="D13" s="58"/>
       <c r="E13" s="33"/>
-      <c r="F13" s="73"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I13" s="72" t="s">
+      <c r="F13" s="107"/>
+      <c r="G13" s="107"/>
+      <c r="H13" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I13" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J13" s="52" t="s">
@@ -2639,7 +2650,7 @@
       <c r="C14" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="99"/>
+      <c r="D14" s="98"/>
       <c r="E14" s="53"/>
       <c r="F14" s="64"/>
       <c r="G14" s="64"/>
@@ -2660,7 +2671,7 @@
       <c r="C15" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="78"/>
+      <c r="D15" s="108"/>
       <c r="E15" s="80"/>
       <c r="F15" s="81"/>
       <c r="G15" s="81"/>
@@ -2673,20 +2684,20 @@
       <c r="C16" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="78"/>
+      <c r="D16" s="108"/>
       <c r="E16" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F16" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G16" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H16" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I16" s="31" t="s">
+      <c r="F16" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G16" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H16" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I16" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J16" s="61" t="s">
@@ -2700,20 +2711,20 @@
       <c r="C17" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="78"/>
+      <c r="D17" s="108"/>
       <c r="E17" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F17" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G17" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H17" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I17" s="31" t="s">
+      <c r="F17" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G17" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I17" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J17" s="61" t="s">
@@ -2727,20 +2738,20 @@
       <c r="C18" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="78"/>
+      <c r="D18" s="108"/>
       <c r="E18" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F18" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G18" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H18" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I18" s="31" t="s">
+      <c r="F18" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H18" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I18" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J18" s="61" t="s">
@@ -2754,20 +2765,20 @@
       <c r="C19" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="78"/>
+      <c r="D19" s="108"/>
       <c r="E19" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F19" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G19" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H19" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I19" s="31" t="s">
+      <c r="F19" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G19" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H19" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I19" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J19" s="61" t="s">
@@ -2781,20 +2792,20 @@
       <c r="C20" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="78"/>
+      <c r="D20" s="108"/>
       <c r="E20" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G20" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H20" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I20" s="31" t="s">
+      <c r="F20" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G20" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H20" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I20" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J20" s="61" t="s">
@@ -2808,20 +2819,20 @@
       <c r="C21" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="78"/>
+      <c r="D21" s="108"/>
       <c r="E21" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F21" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G21" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H21" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I21" s="31" t="s">
+      <c r="F21" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G21" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H21" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I21" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J21" s="61" t="s">
@@ -2835,20 +2846,20 @@
       <c r="C22" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="78"/>
+      <c r="D22" s="108"/>
       <c r="E22" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F22" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G22" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="H22" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I22" s="31" t="s">
+      <c r="F22" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="G22" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="H22" s="109" t="s">
+        <v>0</v>
+      </c>
+      <c r="I22" s="109" t="s">
         <v>0</v>
       </c>
       <c r="J22" s="61" t="s">
@@ -2889,12 +2900,12 @@
       <c r="C24" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="71"/>
+      <c r="D24" s="105"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="71"/>
-      <c r="G24" s="71"/>
-      <c r="H24" s="71"/>
-      <c r="I24" s="71"/>
+      <c r="F24" s="105"/>
+      <c r="G24" s="105"/>
+      <c r="H24" s="105"/>
+      <c r="I24" s="105"/>
       <c r="J24" s="58"/>
       <c r="K24" s="17"/>
     </row>
@@ -2902,20 +2913,20 @@
       <c r="C25" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="71"/>
+      <c r="D25" s="105"/>
       <c r="E25" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F25" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G25" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H25" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I25" s="72" t="s">
+      <c r="F25" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G25" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H25" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I25" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J25" s="52" t="s">
@@ -2929,20 +2940,20 @@
       <c r="C26" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="71"/>
+      <c r="D26" s="105"/>
       <c r="E26" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G26" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H26" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I26" s="72" t="s">
+      <c r="F26" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G26" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H26" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I26" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J26" s="52" t="s">
@@ -2956,20 +2967,20 @@
       <c r="C27" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D27" s="71"/>
+      <c r="D27" s="105"/>
       <c r="E27" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G27" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H27" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I27" s="72" t="s">
+      <c r="F27" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G27" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H27" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I27" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J27" s="52" t="s">
@@ -2983,20 +2994,20 @@
       <c r="C28" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="71"/>
+      <c r="D28" s="105"/>
       <c r="E28" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F28" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="G28" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="H28" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="I28" s="72" t="s">
+      <c r="F28" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="G28" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="H28" s="106" t="s">
+        <v>0</v>
+      </c>
+      <c r="I28" s="106" t="s">
         <v>0</v>
       </c>
       <c r="J28" s="52" t="s">
@@ -3029,8 +3040,8 @@
       <c r="J29" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="K29" s="98" t="s">
-        <v>51</v>
+      <c r="K29" s="110" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Program Exit Survey Updates
</commit_message>
<xml_diff>
--- a/ABET/DocumentTracker_Assessment.xlsx
+++ b/ABET/DocumentTracker_Assessment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usarmywestpoint-my.sharepoint.com/personal/andrew_biaglow_westpoint_edu/Documents/Documents/GitHub/abiaglow.github.io/ABET/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A341C86-E72B-4701-8C4E-954FA9B09F0C}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16C30DEA-8C95-41EC-BD1F-75F6FB2F9DCC}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-72" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -694,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -903,6 +903,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -917,20 +920,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1267,15 +1256,15 @@
     <row r="3" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C3" s="13"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="100" t="s">
+      <c r="E3" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="102"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="103"/>
     </row>
     <row r="4" spans="3:28" x14ac:dyDescent="0.3">
       <c r="C4" s="14"/>
@@ -1301,15 +1290,15 @@
       <c r="K4" s="15">
         <v>2026</v>
       </c>
-      <c r="N4" s="103" t="s">
+      <c r="N4" s="104" t="s">
         <v>48</v>
       </c>
-      <c r="O4" s="104"/>
+      <c r="O4" s="105"/>
       <c r="P4" s="42"/>
-      <c r="R4" s="103" t="s">
+      <c r="R4" s="104" t="s">
         <v>39</v>
       </c>
-      <c r="S4" s="104"/>
+      <c r="S4" s="105"/>
       <c r="T4" s="42"/>
       <c r="V4" s="54" t="s">
         <v>45</v>
@@ -2402,15 +2391,15 @@
     <row r="3" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C3" s="13"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="100" t="s">
+      <c r="E3" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="102"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="103"/>
     </row>
     <row r="4" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C4" s="14"/>
@@ -2441,12 +2430,12 @@
       <c r="C5" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="105"/>
+      <c r="D5" s="71"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="105"/>
-      <c r="G5" s="105"/>
-      <c r="H5" s="105"/>
-      <c r="I5" s="105"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
       <c r="J5" s="58"/>
       <c r="K5" s="17"/>
     </row>
@@ -2454,20 +2443,20 @@
       <c r="C6" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="105"/>
+      <c r="D6" s="71"/>
       <c r="E6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H6" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I6" s="106" t="s">
+      <c r="F6" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I6" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J6" s="52" t="s">
@@ -2481,20 +2470,20 @@
       <c r="C7" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="105"/>
+      <c r="D7" s="71"/>
       <c r="E7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G7" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I7" s="106" t="s">
+      <c r="F7" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H7" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I7" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J7" s="52" t="s">
@@ -2508,27 +2497,27 @@
       <c r="C8" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="105"/>
+      <c r="D8" s="71"/>
       <c r="E8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F8" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G8" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H8" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8" s="106" t="s">
+      <c r="F8" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H8" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I8" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J8" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="K8" s="66" t="s">
-        <v>52</v>
+      <c r="K8" s="70" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="3:11" x14ac:dyDescent="0.3">
@@ -2548,7 +2537,7 @@
       <c r="H9" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="I9" s="106" t="s">
+      <c r="I9" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J9" s="63" t="s">
@@ -2594,7 +2583,7 @@
       <c r="F11" s="51"/>
       <c r="G11" s="51"/>
       <c r="H11" s="51"/>
-      <c r="I11" s="105"/>
+      <c r="I11" s="71"/>
       <c r="J11" s="58"/>
       <c r="K11" s="17"/>
     </row>
@@ -2606,16 +2595,16 @@
       <c r="E12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F12" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G12" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H12" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I12" s="106" t="s">
+      <c r="F12" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H12" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I12" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J12" s="52" t="s">
@@ -2631,12 +2620,12 @@
       </c>
       <c r="D13" s="58"/>
       <c r="E13" s="33"/>
-      <c r="F13" s="107"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I13" s="106" t="s">
+      <c r="F13" s="73"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I13" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J13" s="52" t="s">
@@ -2671,7 +2660,7 @@
       <c r="C15" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="108"/>
+      <c r="D15" s="78"/>
       <c r="E15" s="80"/>
       <c r="F15" s="81"/>
       <c r="G15" s="81"/>
@@ -2684,20 +2673,20 @@
       <c r="C16" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="108"/>
+      <c r="D16" s="78"/>
       <c r="E16" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F16" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G16" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H16" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I16" s="109" t="s">
+      <c r="F16" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H16" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I16" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J16" s="61" t="s">
@@ -2711,20 +2700,20 @@
       <c r="C17" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="108"/>
+      <c r="D17" s="78"/>
       <c r="E17" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F17" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G17" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H17" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I17" s="109" t="s">
+      <c r="F17" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I17" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J17" s="61" t="s">
@@ -2738,20 +2727,20 @@
       <c r="C18" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="108"/>
+      <c r="D18" s="78"/>
       <c r="E18" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F18" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G18" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H18" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I18" s="109" t="s">
+      <c r="F18" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I18" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J18" s="61" t="s">
@@ -2765,20 +2754,20 @@
       <c r="C19" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="108"/>
+      <c r="D19" s="78"/>
       <c r="E19" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F19" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G19" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H19" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I19" s="109" t="s">
+      <c r="F19" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G19" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H19" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I19" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J19" s="61" t="s">
@@ -2792,20 +2781,20 @@
       <c r="C20" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="108"/>
+      <c r="D20" s="78"/>
       <c r="E20" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G20" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H20" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I20" s="109" t="s">
+      <c r="F20" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G20" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H20" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I20" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J20" s="61" t="s">
@@ -2819,20 +2808,20 @@
       <c r="C21" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="108"/>
+      <c r="D21" s="78"/>
       <c r="E21" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F21" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G21" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H21" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I21" s="109" t="s">
+      <c r="F21" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H21" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I21" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J21" s="61" t="s">
@@ -2846,20 +2835,20 @@
       <c r="C22" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="108"/>
+      <c r="D22" s="78"/>
       <c r="E22" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="F22" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="G22" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="H22" s="109" t="s">
-        <v>0</v>
-      </c>
-      <c r="I22" s="109" t="s">
+      <c r="F22" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="H22" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="I22" s="31" t="s">
         <v>0</v>
       </c>
       <c r="J22" s="61" t="s">
@@ -2900,12 +2889,12 @@
       <c r="C24" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="105"/>
+      <c r="D24" s="71"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="105"/>
-      <c r="G24" s="105"/>
-      <c r="H24" s="105"/>
-      <c r="I24" s="105"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71"/>
+      <c r="I24" s="71"/>
       <c r="J24" s="58"/>
       <c r="K24" s="17"/>
     </row>
@@ -2913,20 +2902,20 @@
       <c r="C25" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="D25" s="105"/>
+      <c r="D25" s="71"/>
       <c r="E25" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F25" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G25" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H25" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I25" s="106" t="s">
+      <c r="F25" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G25" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H25" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I25" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J25" s="52" t="s">
@@ -2940,20 +2929,20 @@
       <c r="C26" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="105"/>
+      <c r="D26" s="71"/>
       <c r="E26" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G26" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H26" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I26" s="106" t="s">
+      <c r="F26" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G26" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H26" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I26" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J26" s="52" t="s">
@@ -2967,20 +2956,20 @@
       <c r="C27" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D27" s="105"/>
+      <c r="D27" s="71"/>
       <c r="E27" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F27" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G27" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H27" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I27" s="106" t="s">
+      <c r="F27" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G27" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H27" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I27" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J27" s="52" t="s">
@@ -2994,20 +2983,20 @@
       <c r="C28" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="105"/>
+      <c r="D28" s="71"/>
       <c r="E28" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F28" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="G28" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="H28" s="106" t="s">
-        <v>0</v>
-      </c>
-      <c r="I28" s="106" t="s">
+      <c r="F28" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="G28" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="H28" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="I28" s="72" t="s">
         <v>0</v>
       </c>
       <c r="J28" s="52" t="s">
@@ -3040,7 +3029,7 @@
       <c r="J29" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="K29" s="110" t="s">
+      <c r="K29" s="100" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker with student outcome surveys
</commit_message>
<xml_diff>
--- a/ABET/DocumentTracker_Assessment.xlsx
+++ b/ABET/DocumentTracker_Assessment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usarmywestpoint-my.sharepoint.com/personal/andrew_biaglow_westpoint_edu/Documents/Documents/GitHub/abiaglow.github.io/ABET/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16C30DEA-8C95-41EC-BD1F-75F6FB2F9DCC}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED1D00AC-1A4D-45D8-BA2F-C0D049E46261}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
+    <workbookView xWindow="22932" yWindow="-72" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2462,8 +2462,8 @@
       <c r="J6" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="K6" s="66" t="s">
-        <v>52</v>
+      <c r="K6" s="70" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="3:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added faculty survey results to ABET docs
</commit_message>
<xml_diff>
--- a/ABET/DocumentTracker_Assessment.xlsx
+++ b/ABET/DocumentTracker_Assessment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usarmywestpoint-my.sharepoint.com/personal/andrew_biaglow_westpoint_edu/Documents/Documents/GitHub/abiaglow.github.io/ABET/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7F7AE9-C6A0-4933-848E-B1C9B75C5BB9}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{EFECDF9E-D228-4EC8-8531-E9F428053B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFC065BB-681E-408A-BD3B-14E27C1944F1}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-72" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{188796DA-674F-42F3-8244-EB71C3832B77}"/>
   </bookViews>
@@ -2543,8 +2543,8 @@
       <c r="J9" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="K9" s="67" t="s">
-        <v>53</v>
+      <c r="K9" s="77" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="3:11" x14ac:dyDescent="0.3">

</xml_diff>